<commit_message>
Update Excel IMP status for 18 newly implemented rules
Changed from ⚠️ to ✅:
- Precise, Good Shot, Bad Shot
- Point-Blank Surge, Predator Fighter
- Shielded, Protected, Resistance
- Melee Evasion, Melee Shrouding, Ranged Shrouding
- Morale Boost, No Retreat, Battleborn
- Rapid Charge, Agile, Fast, Slow

Implementation status summary:
- ✅ Fully implemented: 42 rules
- ⚠️ Defined but not implemented: 18 rules
- ❌ Not in code: 456 rules
</commit_message>
<xml_diff>
--- a/docs/special_rules_review_matrix.xlsx
+++ b/docs/special_rules_review_matrix.xlsx
@@ -1004,7 +1004,7 @@
       <c r="U7" t="inlineStr"/>
       <c r="V7" t="inlineStr">
         <is>
-          <t>⚠️</t>
+          <t>✅</t>
         </is>
       </c>
     </row>
@@ -1932,7 +1932,7 @@
       <c r="U19" t="inlineStr"/>
       <c r="V19" t="inlineStr">
         <is>
-          <t>⚠️</t>
+          <t>✅</t>
         </is>
       </c>
     </row>
@@ -2158,7 +2158,7 @@
       <c r="U22" t="inlineStr"/>
       <c r="V22" t="inlineStr">
         <is>
-          <t>⚠️</t>
+          <t>✅</t>
         </is>
       </c>
     </row>
@@ -2236,7 +2236,7 @@
       <c r="U23" t="inlineStr"/>
       <c r="V23" t="inlineStr">
         <is>
-          <t>⚠️</t>
+          <t>✅</t>
         </is>
       </c>
     </row>
@@ -2384,7 +2384,7 @@
       <c r="U25" t="inlineStr"/>
       <c r="V25" t="inlineStr">
         <is>
-          <t>⚠️</t>
+          <t>✅</t>
         </is>
       </c>
     </row>
@@ -2458,7 +2458,7 @@
       <c r="U26" t="inlineStr"/>
       <c r="V26" t="inlineStr">
         <is>
-          <t>⚠️</t>
+          <t>✅</t>
         </is>
       </c>
     </row>
@@ -2532,7 +2532,7 @@
       <c r="U27" t="inlineStr"/>
       <c r="V27" t="inlineStr">
         <is>
-          <t>⚠️</t>
+          <t>✅</t>
         </is>
       </c>
     </row>
@@ -2992,7 +2992,7 @@
       <c r="U33" t="inlineStr"/>
       <c r="V33" t="inlineStr">
         <is>
-          <t>⚠️</t>
+          <t>✅</t>
         </is>
       </c>
     </row>
@@ -3066,7 +3066,7 @@
       <c r="U34" t="inlineStr"/>
       <c r="V34" t="inlineStr">
         <is>
-          <t>⚠️</t>
+          <t>✅</t>
         </is>
       </c>
     </row>
@@ -3140,7 +3140,7 @@
       <c r="U35" t="inlineStr"/>
       <c r="V35" t="inlineStr">
         <is>
-          <t>⚠️</t>
+          <t>✅</t>
         </is>
       </c>
     </row>
@@ -3292,7 +3292,7 @@
       <c r="U37" t="inlineStr"/>
       <c r="V37" t="inlineStr">
         <is>
-          <t>⚠️</t>
+          <t>✅</t>
         </is>
       </c>
     </row>
@@ -4216,7 +4216,7 @@
       <c r="U49" t="inlineStr"/>
       <c r="V49" t="inlineStr">
         <is>
-          <t>⚠️</t>
+          <t>✅</t>
         </is>
       </c>
     </row>
@@ -4294,7 +4294,7 @@
       <c r="U50" t="inlineStr"/>
       <c r="V50" t="inlineStr">
         <is>
-          <t>⚠️</t>
+          <t>✅</t>
         </is>
       </c>
     </row>
@@ -4372,7 +4372,7 @@
       <c r="U51" t="inlineStr"/>
       <c r="V51" t="inlineStr">
         <is>
-          <t>⚠️</t>
+          <t>✅</t>
         </is>
       </c>
     </row>
@@ -4602,7 +4602,7 @@
       <c r="U54" t="inlineStr"/>
       <c r="V54" t="inlineStr">
         <is>
-          <t>⚠️</t>
+          <t>✅</t>
         </is>
       </c>
     </row>
@@ -4676,7 +4676,7 @@
       <c r="U55" t="inlineStr"/>
       <c r="V55" t="inlineStr">
         <is>
-          <t>⚠️</t>
+          <t>✅</t>
         </is>
       </c>
     </row>
@@ -4750,7 +4750,7 @@
       <c r="U56" t="inlineStr"/>
       <c r="V56" t="inlineStr">
         <is>
-          <t>⚠️</t>
+          <t>✅</t>
         </is>
       </c>
     </row>
@@ -4824,7 +4824,7 @@
       <c r="U57" t="inlineStr"/>
       <c r="V57" t="inlineStr">
         <is>
-          <t>⚠️</t>
+          <t>✅</t>
         </is>
       </c>
     </row>

</xml_diff>